<commit_message>
add bin q back in
</commit_message>
<xml_diff>
--- a/docs/form.xlsx
+++ b/docs/form.xlsx
@@ -6791,27 +6791,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -6829,20 +6809,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8604,7 +8570,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>85</v>
@@ -8952,7 +8918,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>100</v>
@@ -19404,8 +19370,6 @@
       <c r="AN295" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B164:B167 B169:B173"/>
-  <conditionalFormatting sqref="B197:B293"/>
   <dataValidations count="30">
     <dataValidation type="list" allowBlank="1" sqref="A165:A167">
       <formula1>QuestionTypes</formula1>
@@ -21404,20 +21368,20 @@
   <sheetPr>
     <tabColor theme="4" tint="0.3999755851924192"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="8.85546875"/>
   <cols>
     <col min="1" max="1" width="52.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.95" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="48" t="s">
         <v>481</v>
       </c>
       <c r="B1"/>
     </row>
-    <row r="2" ht="15.95" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="49"/>
       <c r="B2" s="49"/>
     </row>
@@ -23142,10 +23106,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:E39">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"No"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24806,8 +24770,6 @@
     <mergeCell ref="D35:D37"/>
     <mergeCell ref="D40:D41"/>
   </mergeCells>
-  <conditionalFormatting sqref="B29"/>
-  <conditionalFormatting sqref="B30:B44"/>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1"/>
     <hyperlink ref="D8" r:id="rId2"/>

</xml_diff>